<commit_message>
Update real contact info in contacto.html and Excel
- Email: morenosantosjoiers@gmail.com (replaces Cloudflare-obfuscated placeholder)
- Phone: +34 93 219 00 11 (replaces fake +34 932 000 000)
- WhatsApp: +34 93 219 00 11 same number (replaces fake +34 600 000 000)
- Address: Carrer de l'Escorial, 162, Local 2 · Barcelona 08024
  (replaces fictional Carrer del Bisbe, 12 · Barrio Gótico)
- Google Maps link updated with real address
- Excel updated to reflect these changes

https://claude.ai/code/session_01JHX15pgbNp5TiuNNpfm5mN
</commit_message>
<xml_diff>
--- a/textos_web_moreno_santos.xlsx
+++ b/textos_web_moreno_santos.xlsx
@@ -3427,17 +3427,17 @@
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>[email protected]</t>
+          <t>[email protected] (ofuscado Cloudflare)</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>[email real de Moreno Santos Joiers]</t>
+          <t>morenosantosjoiers@gmail.com</t>
         </is>
       </c>
       <c r="F92" s="6" t="inlineStr">
         <is>
-          <t>Actualizar con el email real de la empresa.</t>
+          <t>Email real actualizado en el HTML. Enlace mailto: funcional.</t>
         </is>
       </c>
     </row>
@@ -3464,12 +3464,12 @@
       </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
-          <t>[Teléfono real de Moreno Santos Joiers]</t>
+          <t>+34 93 219 00 11</t>
         </is>
       </c>
       <c r="F93" s="6" t="inlineStr">
         <is>
-          <t>Actualizar con el teléfono real de la empresa.</t>
+          <t>Teléfono real actualizado en el HTML con href tel:+34932190011.</t>
         </is>
       </c>
     </row>
@@ -3496,12 +3496,12 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t>[WhatsApp real de Moreno Santos Joiers]</t>
+          <t>+34 93 219 00 11</t>
         </is>
       </c>
       <c r="F94" s="6" t="inlineStr">
         <is>
-          <t>Actualizar con el WhatsApp real si disponéis de él.</t>
+          <t>Mismo número que teléfono. Actualizado en el HTML con href wa.me/34932190011.</t>
         </is>
       </c>
     </row>
@@ -3747,17 +3747,17 @@
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Carrer del Bisbe, 12</t>
+          <t>Carrer del Bisbe, 12 · Barrio Gótico, Barcelona 08002</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t>[Dirección real de Moreno Santos Joiers]</t>
+          <t>Carrer de l'Escorial, 162, Local 2 · Barcelona 08024</t>
         </is>
       </c>
       <c r="F102" s="6" t="inlineStr">
         <is>
-          <t>Actualizar con dirección real.</t>
+          <t>Dirección real actualizada en el HTML.</t>
         </is>
       </c>
     </row>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>Metro</t>
+          <t>Metro / barrio</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -3784,12 +3784,12 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>[Indicaciones de transporte real]</t>
+          <t>Barcelona 08024 · Local 2</t>
         </is>
       </c>
       <c r="F103" s="6" t="inlineStr">
         <is>
-          <t>Actualizar con indicaciones reales.</t>
+          <t>Actualizado en el mapa del HTML. Añadir indicaciones de metro/bus si procede.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel with WhatsApp pre-filled message entry
https://claude.ai/code/session_01JHX15pgbNp5TiuNNpfm5mN
</commit_message>
<xml_diff>
--- a/textos_web_moreno_santos.xlsx
+++ b/textos_web_moreno_santos.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F116"/>
+  <dimension ref="A1:F117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3513,27 +3513,27 @@
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>Formulario</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>Título</t>
+          <t>Mensaje prellenado</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Escríbenos lo que necesitas</t>
+          <t>Hola, me gustaría obtener más información.</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>Escríbenos — Te respondemos en menos de 24h</t>
+          <t>Hola, he visto vuestra página web y quería pediros información sobre</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>Añadir tiempo de respuesta en el título para generar confianza.</t>
+          <t>Actualizado. El usuario completa la frase antes de enviar.</t>
         </is>
       </c>
     </row>
@@ -3550,22 +3550,22 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Opción dropdown 1</t>
+          <t>Título</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>Información sobre una pieza</t>
+          <t>Escríbenos lo que necesitas</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t>Información sobre una joya</t>
+          <t>Escríbenos — Te respondemos en menos de 24h</t>
         </is>
       </c>
       <c r="F96" s="6" t="inlineStr">
         <is>
-          <t>Usar 'joya' en lugar de 'pieza'.</t>
+          <t>Añadir tiempo de respuesta en el título para generar confianza.</t>
         </is>
       </c>
     </row>
@@ -3582,22 +3582,22 @@
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>Opción dropdown 2</t>
+          <t>Opción dropdown 1</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>Encargo personal</t>
+          <t>Información sobre una pieza</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t>Quiero crear una joya a medida</t>
+          <t>Información sobre una joya</t>
         </is>
       </c>
       <c r="F97" s="6" t="inlineStr">
         <is>
-          <t>Más descriptivo y accionable.</t>
+          <t>Usar 'joya' en lugar de 'pieza'.</t>
         </is>
       </c>
     </row>
@@ -3614,22 +3614,22 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Opción dropdown 3</t>
+          <t>Opción dropdown 2</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Visita al atelier</t>
+          <t>Encargo personal</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>Quiero visitar el taller</t>
+          <t>Quiero crear una joya a medida</t>
         </is>
       </c>
       <c r="F98" s="6" t="inlineStr">
         <is>
-          <t>Usar 'taller' en lugar de 'atelier'.</t>
+          <t>Más descriptivo y accionable.</t>
         </is>
       </c>
     </row>
@@ -3646,22 +3646,22 @@
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>Opción dropdown 4</t>
+          <t>Opción dropdown 3</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>Reparación o mantenimiento</t>
+          <t>Visita al atelier</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t>Reparación de joya o reloj</t>
+          <t>Quiero visitar el taller</t>
         </is>
       </c>
       <c r="F99" s="6" t="inlineStr">
         <is>
-          <t>Añadir 'reloj' ya que también reparáis relojería.</t>
+          <t>Usar 'taller' en lugar de 'atelier'.</t>
         </is>
       </c>
     </row>
@@ -3678,22 +3678,22 @@
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Opción dropdown 5</t>
+          <t>Opción dropdown 4</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Colaboración o prensa</t>
+          <t>Reparación o mantenimiento</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t>Colaboración o prensa</t>
+          <t>Reparación de joya o reloj</t>
         </is>
       </c>
       <c r="F100" s="6" t="inlineStr">
         <is>
-          <t>Mantener si aplica.</t>
+          <t>Añadir 'reloj' ya que también reparáis relojería.</t>
         </is>
       </c>
     </row>
@@ -3710,22 +3710,22 @@
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>Opción dropdown 6</t>
+          <t>Opción dropdown 5</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>[No existe]</t>
+          <t>Colaboración o prensa</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>Grabación personalizada</t>
+          <t>Colaboración o prensa</t>
         </is>
       </c>
       <c r="F101" s="6" t="inlineStr">
         <is>
-          <t>Añadir opción para el servicio de grabaciones.</t>
+          <t>Mantener si aplica.</t>
         </is>
       </c>
     </row>
@@ -3737,27 +3737,27 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Ubicación</t>
+          <t>Formulario</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>Dirección</t>
+          <t>Opción dropdown 6</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Carrer del Bisbe, 12 · Barrio Gótico, Barcelona 08002</t>
+          <t>[No existe]</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t>Carrer de l'Escorial, 162, Local 2 · Barcelona 08024</t>
+          <t>Grabación personalizada</t>
         </is>
       </c>
       <c r="F102" s="6" t="inlineStr">
         <is>
-          <t>Dirección real actualizada en el HTML.</t>
+          <t>Añadir opción para el servicio de grabaciones.</t>
         </is>
       </c>
     </row>
@@ -3774,22 +3774,22 @@
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>Metro / barrio</t>
+          <t>Dirección</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>Barrio Gótico · Metro Jaume I (L4)</t>
+          <t>Carrer del Bisbe, 12 · Barrio Gótico, Barcelona 08002</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>Barcelona 08024 · Local 2</t>
+          <t>Carrer de l'Escorial, 162, Local 2 · Barcelona 08024</t>
         </is>
       </c>
       <c r="F103" s="6" t="inlineStr">
         <is>
-          <t>Actualizado en el mapa del HTML. Añadir indicaciones de metro/bus si procede.</t>
+          <t>Dirección real actualizada en el HTML.</t>
         </is>
       </c>
     </row>
@@ -3801,27 +3801,27 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Horarios</t>
+          <t>Ubicación</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Lunes-Viernes</t>
+          <t>Metro / barrio</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>10:00 – 19:00</t>
+          <t>Barrio Gótico · Metro Jaume I (L4)</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t>[Horario real de apertura]</t>
+          <t>Barcelona 08024 · Local 2</t>
         </is>
       </c>
       <c r="F104" s="6" t="inlineStr">
         <is>
-          <t>Actualizar con horario real.</t>
+          <t>Actualizado en el mapa del HTML. Añadir indicaciones de metro/bus si procede.</t>
         </is>
       </c>
     </row>
@@ -3838,17 +3838,17 @@
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Lunes-Viernes</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>11:00 – 18:00</t>
+          <t>10:00 – 19:00</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>[Horario real de sábado]</t>
+          <t>[Horario real de apertura]</t>
         </is>
       </c>
       <c r="F105" s="6" t="inlineStr">
@@ -3865,59 +3865,59 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Servicios</t>
+          <t>Horarios</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Reparaciones</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>Aceptamos joyas de otras marcas. Consulta disponibilidad y presupuesto sin compromiso.</t>
+          <t>11:00 – 18:00</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>Reparamos y restauramos joyas y relojes de cualquier marca. Consulta sin compromiso.</t>
+          <t>[Horario real de sábado]</t>
         </is>
       </c>
       <c r="F106" s="6" t="inlineStr">
         <is>
-          <t>Añadir 'relojes' explícitamente.</t>
+          <t>Actualizar con horario real.</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Contacto</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
         <is>
-          <t>Navegación</t>
+          <t>Servicios</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>Item 1</t>
+          <t>Reparaciones</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>Colecciones</t>
+          <t>Aceptamos joyas de otras marcas. Consulta disponibilidad y presupuesto sin compromiso.</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t>Colecciones</t>
+          <t>Reparamos y restauramos joyas y relojes de cualquier marca. Consulta sin compromiso.</t>
         </is>
       </c>
       <c r="F107" s="6" t="inlineStr">
         <is>
-          <t>Correcto.</t>
+          <t>Añadir 'relojes' explícitamente.</t>
         </is>
       </c>
     </row>
@@ -3934,22 +3934,22 @@
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>Item 2</t>
+          <t>Item 1</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>Atelier</t>
+          <t>Colecciones</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>Taller</t>
+          <t>Colecciones</t>
         </is>
       </c>
       <c r="F108" s="6" t="inlineStr">
         <is>
-          <t>Usar 'Taller' es más natural en español/catalán para empresa familiar.</t>
+          <t>Correcto.</t>
         </is>
       </c>
     </row>
@@ -3966,22 +3966,22 @@
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>Item 3</t>
+          <t>Item 2</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>Encargo</t>
+          <t>Atelier</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>Encargo a medida</t>
+          <t>Taller</t>
         </is>
       </c>
       <c r="F109" s="6" t="inlineStr">
         <is>
-          <t>Más descriptivo.</t>
+          <t>Usar 'Taller' es más natural en español/catalán para empresa familiar.</t>
         </is>
       </c>
     </row>
@@ -3998,22 +3998,22 @@
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>Item 4</t>
+          <t>Item 3</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Nosotros</t>
+          <t>Encargo</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>Nosotros</t>
+          <t>Encargo a medida</t>
         </is>
       </c>
       <c r="F110" s="6" t="inlineStr">
         <is>
-          <t>Correcto.</t>
+          <t>Más descriptivo.</t>
         </is>
       </c>
     </row>
@@ -4030,17 +4030,17 @@
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>Item 5</t>
+          <t>Item 4</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>Contacto</t>
+          <t>Nosotros</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>Contacto</t>
+          <t>Nosotros</t>
         </is>
       </c>
       <c r="F111" s="6" t="inlineStr">
@@ -4057,27 +4057,27 @@
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>Redes sociales</t>
+          <t>Navegación</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>Instagram handle</t>
+          <t>Item 5</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>@morenosantos</t>
+          <t>Contacto</t>
         </is>
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t>[Handle real de Instagram de Moreno Santos Joiers]</t>
+          <t>Contacto</t>
         </is>
       </c>
       <c r="F112" s="6" t="inlineStr">
         <is>
-          <t>Actualizar con cuenta real.</t>
+          <t>Correcto.</t>
         </is>
       </c>
     </row>
@@ -4094,22 +4094,22 @@
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>Pinterest</t>
+          <t>Instagram handle</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>Moreno Santos</t>
+          <t>@morenosantos</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t>[Cuenta real de Pinterest si existe]</t>
+          <t>[Handle real de Instagram de Moreno Santos Joiers]</t>
         </is>
       </c>
       <c r="F113" s="6" t="inlineStr">
         <is>
-          <t>Verificar si tenéis Pinterest activo.</t>
+          <t>Actualizar con cuenta real.</t>
         </is>
       </c>
     </row>
@@ -4121,27 +4121,27 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>Footer links</t>
+          <t>Redes sociales</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>Privacidad</t>
+          <t>Pinterest</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>Privacidad</t>
+          <t>Moreno Santos</t>
         </is>
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t>Política de privacidad</t>
+          <t>[Cuenta real de Pinterest si existe]</t>
         </is>
       </c>
       <c r="F114" s="6" t="inlineStr">
         <is>
-          <t>Texto completo es más claro para el usuario.</t>
+          <t>Verificar si tenéis Pinterest activo.</t>
         </is>
       </c>
     </row>
@@ -4158,22 +4158,22 @@
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Privacidad</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>Envíos</t>
+          <t>Privacidad</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
         <is>
-          <t>Envíos y devoluciones</t>
+          <t>Política de privacidad</t>
         </is>
       </c>
       <c r="F115" s="6" t="inlineStr">
         <is>
-          <t>Ampliar si también tenéis política de devoluciones.</t>
+          <t>Texto completo es más claro para el usuario.</t>
         </is>
       </c>
     </row>
@@ -4185,25 +4185,57 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
+          <t>Footer links</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>Envíos</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>Envíos</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>Envíos y devoluciones</t>
+        </is>
+      </c>
+      <c r="F116" s="6" t="inlineStr">
+        <is>
+          <t>Ampliar si también tenéis política de devoluciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="15" customHeight="1">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
           <t>Meta / SEO</t>
         </is>
       </c>
-      <c r="C116" s="3" t="inlineStr">
+      <c r="C117" s="7" t="inlineStr">
         <is>
           <t>Descripción general</t>
         </is>
       </c>
-      <c r="D116" s="4" t="inlineStr">
+      <c r="D117" s="4" t="inlineStr">
         <is>
           <t>[No definida en el código]</t>
         </is>
       </c>
-      <c r="E116" s="5" t="inlineStr">
+      <c r="E117" s="5" t="inlineStr">
         <is>
           <t>Joyería artesanal en Barcelona desde 1993. Diseños propios en oro de 18 quilates, diamantes y piedras preciosas. Taller propio, alianzas de boda, reparaciones y grabaciones.</t>
         </is>
       </c>
-      <c r="F116" s="6" t="inlineStr">
+      <c r="F117" s="6" t="inlineStr">
         <is>
           <t>Añadir meta description en todas las páginas para mejorar el SEO.</t>
         </is>

</xml_diff>